<commit_message>
Tearsheet README: TWR / IRR / risk stats vs KOSPI, monthly returns, attribution, execution; monthly NAV data
</commit_message>
<xml_diff>
--- a/data/Kiwoom_Transactions.xlsx
+++ b/data/Kiwoom_Transactions.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Year" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Stock" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trades" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holdings" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Transactions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly NAV" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Stock" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trades" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holdings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Transactions" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,9 +23,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0;[Red]-#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%;[Red]-0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -85,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -103,6 +106,15 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -468,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -516,7 +528,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>95600000</v>
+        <v>95000000</v>
       </c>
     </row>
     <row r="7">
@@ -526,7 +538,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>157479843</v>
+        <v>156879843</v>
       </c>
     </row>
     <row r="8">
@@ -556,7 +568,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>176595170</v>
+        <v>175995170</v>
       </c>
     </row>
     <row r="11">
@@ -566,7 +578,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>2.680368052830254</v>
+        <v>2.671261230533257</v>
       </c>
     </row>
     <row r="12">
@@ -589,7 +601,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>22601414.76425532</v>
+        <v>22001414.76425532</v>
       </c>
     </row>
     <row r="15">
@@ -675,6 +687,76 @@
         <is>
           <t>13 / 28</t>
         </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Time-weighted CAGR</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>0.3430717191118919</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>KOSPI CAGR (same window)</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n">
+        <v>0.1512706252547324</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Annualized volatility</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>0.3347163418394256</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sharpe (rf 3%)</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="n">
+        <v>0.9353344309136918</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Max drawdown</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>-0.319880137445345</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Beta to KOSPI</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="n">
+        <v>0.7305380915610608</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Jensen alpha</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>0.2244789079758831</v>
       </c>
     </row>
   </sheetData>
@@ -1046,6 +1128,2158 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Month end</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>Positions</t>
+        </is>
+      </c>
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>Net flow</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>Account return (TWR)</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>KOSPI return</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>Account index</t>
+        </is>
+      </c>
+      <c r="I1" s="17" t="inlineStr">
+        <is>
+          <t>KOSPI index</t>
+        </is>
+      </c>
+      <c r="J1" s="17" t="inlineStr">
+        <is>
+          <t>Equity exposure</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2021-10-31</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="n">
+        <v>65884672</v>
+      </c>
+      <c r="C2" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="18" t="n">
+        <v>65884672</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="19" t="n">
+        <v>-0.01197989973186364</v>
+      </c>
+      <c r="H2" s="20" t="n">
+        <v>100</v>
+      </c>
+      <c r="I2" s="20" t="n">
+        <v>98.80201002681363</v>
+      </c>
+      <c r="J2" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2021-11-30</t>
+        </is>
+      </c>
+      <c r="B3" s="18" t="n">
+        <v>43801362</v>
+      </c>
+      <c r="C3" s="18" t="n">
+        <v>19620000</v>
+      </c>
+      <c r="D3" s="18" t="n">
+        <v>63421362</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="19" t="n">
+        <v>-0.03738821072069692</v>
+      </c>
+      <c r="G3" s="19" t="n">
+        <v>-0.02659334268609925</v>
+      </c>
+      <c r="H3" s="20" t="n">
+        <v>96.26117892793032</v>
+      </c>
+      <c r="I3" s="20" t="n">
+        <v>96.17453431609516</v>
+      </c>
+      <c r="J3" s="21" t="n">
+        <v>0.3093594867924785</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2021-12-31</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="n">
+        <v>43801362</v>
+      </c>
+      <c r="C4" s="18" t="n">
+        <v>20440000</v>
+      </c>
+      <c r="D4" s="18" t="n">
+        <v>64241362</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>0.01292939751120451</v>
+      </c>
+      <c r="G4" s="19" t="n">
+        <v>0.02687498531857502</v>
+      </c>
+      <c r="H4" s="20" t="n">
+        <v>97.50577797518672</v>
+      </c>
+      <c r="I4" s="20" t="n">
+        <v>98.759223513861</v>
+      </c>
+      <c r="J4" s="21" t="n">
+        <v>0.3181750723155589</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2022-01-31</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>43822094</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>20360000</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>64182094</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>-0.0009225831793541364</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>-0.1055563362924995</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>97.41582078453696</v>
+      </c>
+      <c r="I5" s="20" t="n">
+        <v>88.33456170464576</v>
+      </c>
+      <c r="J5" s="21" t="n">
+        <v>0.3172224327863157</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2022-02-28</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>43822094</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>21120000</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>64942094</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>0.0118413088859332</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>0.01345672823119837</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <v>98.56935160882338</v>
+      </c>
+      <c r="I6" s="20" t="n">
+        <v>89.5232558949272</v>
+      </c>
+      <c r="J6" s="21" t="n">
+        <v>0.3252127964952901</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2022-03-31</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>43822094</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>23600000</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>67422094</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>0.03818786625512876</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>0.01506760091792203</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>102.3335048249159</v>
+      </c>
+      <c r="I7" s="20" t="n">
+        <v>90.87215658762497</v>
+      </c>
+      <c r="J7" s="21" t="n">
+        <v>0.3500336254759456</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2022-04-30</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>44517418</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>23040000</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>67557418</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>0.002007116539572325</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>-0.01635127734413222</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>102.5389000950024</v>
+      </c>
+      <c r="I8" s="20" t="n">
+        <v>89.3862807524013</v>
+      </c>
+      <c r="J8" s="21" t="n">
+        <v>0.3410432293312335</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2022-05-31</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>44517418</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>23800000</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>68317418</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>0.01124968985641222</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>-0.003395167554811729</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>103.6924309192888</v>
+      </c>
+      <c r="I9" s="20" t="n">
+        <v>89.08279935214546</v>
+      </c>
+      <c r="J9" s="21" t="n">
+        <v>0.348373821738989</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2022-06-30</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="n">
+        <v>44517418</v>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>19240000</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>63757418</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>-0.06674725324074747</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>-0.1416582874651205</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>96.77124597357033</v>
+      </c>
+      <c r="I10" s="20" t="n">
+        <v>76.46348255332158</v>
+      </c>
+      <c r="J10" s="21" t="n">
+        <v>0.3017688075135038</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2022-07-31</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>44536205</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>19480000</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>64016205</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>0.00405893162110172</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>0.06368908185957856</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <v>97.16403384386587</v>
+      </c>
+      <c r="I11" s="20" t="n">
+        <v>81.33337155292854</v>
+      </c>
+      <c r="J11" s="21" t="n">
+        <v>0.3042979508079243</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2022-08-31</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="n">
+        <v>26353485</v>
+      </c>
+      <c r="C12" s="18" t="n">
+        <v>45080000</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>71433485</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>0.1158656624521869</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>-0.01494133655953711</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <v>108.4220089917121</v>
+      </c>
+      <c r="I12" s="20" t="n">
+        <v>80.11814227503434</v>
+      </c>
+      <c r="J12" s="21" t="n">
+        <v>0.6310765882414948</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2022-09-30</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n">
+        <v>26353485</v>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>41650000</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>68003485</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>-0.04801669693141809</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>-0.1076829892325298</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <v>103.2159422452616</v>
+      </c>
+      <c r="I13" s="20" t="n">
+        <v>71.49078122310154</v>
+      </c>
+      <c r="J13" s="21" t="n">
+        <v>0.6124686109836871</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2022-10-31</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>26371612</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>43820000</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>70191612</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>0.03217668917997364</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>0.08338242408131391</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <v>106.5370895373055</v>
+      </c>
+      <c r="I14" s="20" t="n">
+        <v>77.45185586095062</v>
+      </c>
+      <c r="J14" s="21" t="n">
+        <v>0.6242911190015126</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2022-11-30</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>26371612</v>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>43890000</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>70261612</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>0.0009972701581493811</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>0.06192997619147445</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>106.6433357974371</v>
+      </c>
+      <c r="I15" s="20" t="n">
+        <v>82.2484474504048</v>
+      </c>
+      <c r="J15" s="21" t="n">
+        <v>0.6246654289685241</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2022-12-31</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>26371612</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>39480000</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>65851612</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <v>-0.06276542587722013</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>-0.09816769506050993</v>
+      </c>
+      <c r="H16" s="20" t="n">
+        <v>99.9498214091436</v>
+      </c>
+      <c r="I16" s="20" t="n">
+        <v>74.17430694189308</v>
+      </c>
+      <c r="J16" s="21" t="n">
+        <v>0.5995297427191304</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>26385519</v>
+      </c>
+      <c r="C17" s="18" t="n">
+        <v>37870000</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>64255519</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>-0.02423772101433143</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>0.09542128233002134</v>
+      </c>
+      <c r="H17" s="20" t="n">
+        <v>97.52726552239652</v>
+      </c>
+      <c r="I17" s="20" t="n">
+        <v>81.25211442622911</v>
+      </c>
+      <c r="J17" s="21" t="n">
+        <v>0.5893657165853722</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2023-02-28</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="n">
+        <v>26385519</v>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>40880000</v>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>67265519</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>0.04684422516297783</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>-0.01508284367516044</v>
+      </c>
+      <c r="H18" s="20" t="n">
+        <v>102.0958547080572</v>
+      </c>
+      <c r="I18" s="20" t="n">
+        <v>80.02660148606205</v>
+      </c>
+      <c r="J18" s="21" t="n">
+        <v>0.6077407951018708</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2023-03-31</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n">
+        <v>27569919</v>
+      </c>
+      <c r="C19" s="18" t="n">
+        <v>38710000</v>
+      </c>
+      <c r="D19" s="18" t="n">
+        <v>66279919</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <v>-0.01465238081341497</v>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>0.02652879672375907</v>
+      </c>
+      <c r="H19" s="20" t="n">
+        <v>100.5999073654037</v>
+      </c>
+      <c r="I19" s="20" t="n">
+        <v>82.14961092937907</v>
+      </c>
+      <c r="J19" s="21" t="n">
+        <v>0.5840381307647645</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2023-04-30</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="n">
+        <v>27583905</v>
+      </c>
+      <c r="C20" s="18" t="n">
+        <v>35910000</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <v>63493905</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <v>-0.04203405861132691</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>0.009960159558901616</v>
+      </c>
+      <c r="H20" s="20" t="n">
+        <v>96.37128496291221</v>
+      </c>
+      <c r="I20" s="20" t="n">
+        <v>82.96783416193738</v>
+      </c>
+      <c r="J20" s="21" t="n">
+        <v>0.5655660964623297</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2023-05-31</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="n">
+        <v>27583905</v>
+      </c>
+      <c r="C21" s="18" t="n">
+        <v>33005000</v>
+      </c>
+      <c r="D21" s="18" t="n">
+        <v>60588905</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <v>-0.04575242300816118</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>0.02703940859632104</v>
+      </c>
+      <c r="H21" s="20" t="n">
+        <v>91.96206516744901</v>
+      </c>
+      <c r="I21" s="20" t="n">
+        <v>85.2112353301938</v>
+      </c>
+      <c r="J21" s="21" t="n">
+        <v>0.5447366972550503</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2023-06-30</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="n">
+        <v>27583905</v>
+      </c>
+      <c r="C22" s="18" t="n">
+        <v>34125000</v>
+      </c>
+      <c r="D22" s="18" t="n">
+        <v>61708905</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <v>0.0184852325685701</v>
+      </c>
+      <c r="G22" s="19" t="n">
+        <v>-0.001903296678234634</v>
+      </c>
+      <c r="H22" s="20" t="n">
+        <v>93.6620053295553</v>
+      </c>
+      <c r="I22" s="20" t="n">
+        <v>85.04905306904156</v>
+      </c>
+      <c r="J22" s="21" t="n">
+        <v>0.5529996035418226</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2023-07-31</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="n">
+        <v>127268</v>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>60560500</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>60687768</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="19" t="n">
+        <v>-0.01654764413661205</v>
+      </c>
+      <c r="G23" s="19" t="n">
+        <v>0.04008534087078042</v>
+      </c>
+      <c r="H23" s="20" t="n">
+        <v>92.11211979624035</v>
+      </c>
+      <c r="I23" s="20" t="n">
+        <v>88.45827335205119</v>
+      </c>
+      <c r="J23" s="21" t="n">
+        <v>0.9979029052444308</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2023-08-31</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="n">
+        <v>719468</v>
+      </c>
+      <c r="C24" s="18" t="n">
+        <v>57845000</v>
+      </c>
+      <c r="D24" s="18" t="n">
+        <v>58564468</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="19" t="n">
+        <v>-0.03498728112722814</v>
+      </c>
+      <c r="G24" s="19" t="n">
+        <v>-0.03875417772036871</v>
+      </c>
+      <c r="H24" s="20" t="n">
+        <v>88.88936716570439</v>
+      </c>
+      <c r="I24" s="20" t="n">
+        <v>85.03014570572886</v>
+      </c>
+      <c r="J24" s="21" t="n">
+        <v>0.9877149400554616</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2023-09-30</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="n">
+        <v>719468</v>
+      </c>
+      <c r="C25" s="18" t="n">
+        <v>55282000</v>
+      </c>
+      <c r="D25" s="18" t="n">
+        <v>56001468</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="19" t="n">
+        <v>-0.04376373742522514</v>
+      </c>
+      <c r="G25" s="19" t="n">
+        <v>-0.03847544928290336</v>
+      </c>
+      <c r="H25" s="20" t="n">
+        <v>84.99923624117007</v>
+      </c>
+      <c r="I25" s="20" t="n">
+        <v>81.7585726471102</v>
+      </c>
+      <c r="J25" s="21" t="n">
+        <v>0.9871526939258092</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2023-10-31</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="n">
+        <v>720332</v>
+      </c>
+      <c r="C26" s="18" t="n">
+        <v>47863000</v>
+      </c>
+      <c r="D26" s="18" t="n">
+        <v>48583332</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="19" t="n">
+        <v>-0.1324632418564456</v>
+      </c>
+      <c r="G26" s="19" t="n">
+        <v>-0.06633077569046508</v>
+      </c>
+      <c r="H26" s="20" t="n">
+        <v>73.73996185334281</v>
+      </c>
+      <c r="I26" s="20" t="n">
+        <v>76.33546310408215</v>
+      </c>
+      <c r="J26" s="21" t="n">
+        <v>0.9851732688898325</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2023-11-30</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="n">
+        <v>720332</v>
+      </c>
+      <c r="C27" s="18" t="n">
+        <v>57354000</v>
+      </c>
+      <c r="D27" s="18" t="n">
+        <v>58074332</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="19" t="n">
+        <v>0.1953550653956793</v>
+      </c>
+      <c r="G27" s="19" t="n">
+        <v>0.08839654234188554</v>
+      </c>
+      <c r="H27" s="20" t="n">
+        <v>88.14543692347748</v>
+      </c>
+      <c r="I27" s="20" t="n">
+        <v>83.08325410054958</v>
+      </c>
+      <c r="J27" s="21" t="n">
+        <v>0.9875963790681226</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2023-12-31</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="n">
+        <v>720332</v>
+      </c>
+      <c r="C28" s="18" t="n">
+        <v>57420000</v>
+      </c>
+      <c r="D28" s="18" t="n">
+        <v>58140332</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="19" t="n">
+        <v>0.001136474544382189</v>
+      </c>
+      <c r="G28" s="19" t="n">
+        <v>0.0599877920429186</v>
+      </c>
+      <c r="H28" s="20" t="n">
+        <v>88.24561196874447</v>
+      </c>
+      <c r="I28" s="20" t="n">
+        <v>88.06723506978233</v>
+      </c>
+      <c r="J28" s="21" t="n">
+        <v>0.9876104594655566</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2024-01-31</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="n">
+        <v>722062</v>
+      </c>
+      <c r="C29" s="18" t="n">
+        <v>51593000</v>
+      </c>
+      <c r="D29" s="18" t="n">
+        <v>52315062</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="19" t="n">
+        <v>-0.1001932703101867</v>
+      </c>
+      <c r="G29" s="19" t="n">
+        <v>-0.0424889529972664</v>
+      </c>
+      <c r="H29" s="20" t="n">
+        <v>79.4039955150722</v>
+      </c>
+      <c r="I29" s="20" t="n">
+        <v>84.32535045830313</v>
+      </c>
+      <c r="J29" s="21" t="n">
+        <v>0.9861978181350526</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2024-02-29</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="n">
+        <v>722062</v>
+      </c>
+      <c r="C30" s="18" t="n">
+        <v>52211500</v>
+      </c>
+      <c r="D30" s="18" t="n">
+        <v>52933562</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="19" t="n">
+        <v>0.01182259900599946</v>
+      </c>
+      <c r="G30" s="19" t="n">
+        <v>0.03929271179064631</v>
+      </c>
+      <c r="H30" s="20" t="n">
+        <v>80.34275711352107</v>
+      </c>
+      <c r="I30" s="20" t="n">
+        <v>87.63872215050648</v>
+      </c>
+      <c r="J30" s="21" t="n">
+        <v>0.9863590891540607</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2024-03-31</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="n">
+        <v>722062</v>
+      </c>
+      <c r="C31" s="18" t="n">
+        <v>53388000</v>
+      </c>
+      <c r="D31" s="18" t="n">
+        <v>54110062</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="19" t="n">
+        <v>0.02222597451499674</v>
+      </c>
+      <c r="G31" s="19" t="n">
+        <v>0.0399264277808582</v>
+      </c>
+      <c r="H31" s="20" t="n">
+        <v>82.12845318559077</v>
+      </c>
+      <c r="I31" s="20" t="n">
+        <v>91.13782326125536</v>
+      </c>
+      <c r="J31" s="21" t="n">
+        <v>0.9866556796774693</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2024-04-30</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="n">
+        <v>871743</v>
+      </c>
+      <c r="C32" s="18" t="n">
+        <v>58909500</v>
+      </c>
+      <c r="D32" s="18" t="n">
+        <v>59781243</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="19" t="n">
+        <v>0.1048082517443798</v>
+      </c>
+      <c r="G32" s="19" t="n">
+        <v>-0.02030672838017156</v>
+      </c>
+      <c r="H32" s="20" t="n">
+        <v>90.73619278244267</v>
+      </c>
+      <c r="I32" s="20" t="n">
+        <v>89.28711223912897</v>
+      </c>
+      <c r="J32" s="21" t="n">
+        <v>0.9854177839694634</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2024-05-31</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="n">
+        <v>871743</v>
+      </c>
+      <c r="C33" s="18" t="n">
+        <v>58342000</v>
+      </c>
+      <c r="D33" s="18" t="n">
+        <v>59213743</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="19" t="n">
+        <v>-0.009492944132995026</v>
+      </c>
+      <c r="G33" s="19" t="n">
+        <v>-0.02063105497412732</v>
+      </c>
+      <c r="H33" s="20" t="n">
+        <v>89.87483917351827</v>
+      </c>
+      <c r="I33" s="20" t="n">
+        <v>87.44502491804242</v>
+      </c>
+      <c r="J33" s="21" t="n">
+        <v>0.9852780291223948</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2024-06-30</t>
+        </is>
+      </c>
+      <c r="B34" s="18" t="n">
+        <v>871743</v>
+      </c>
+      <c r="C34" s="18" t="n">
+        <v>65966000</v>
+      </c>
+      <c r="D34" s="18" t="n">
+        <v>66837743</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="19" t="n">
+        <v>0.1287538941762219</v>
+      </c>
+      <c r="G34" s="19" t="n">
+        <v>0.06364072255075515</v>
+      </c>
+      <c r="H34" s="20" t="n">
+        <v>101.4465747055704</v>
+      </c>
+      <c r="I34" s="20" t="n">
+        <v>93.01008948729543</v>
+      </c>
+      <c r="J34" s="21" t="n">
+        <v>0.9869573243967859</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2024-07-31</t>
+        </is>
+      </c>
+      <c r="B35" s="18" t="n">
+        <v>873685</v>
+      </c>
+      <c r="C35" s="18" t="n">
+        <v>83455000</v>
+      </c>
+      <c r="D35" s="18" t="n">
+        <v>84328685</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="19" t="n">
+        <v>0.2616925888715302</v>
+      </c>
+      <c r="G35" s="19" t="n">
+        <v>-0.009496142151442011</v>
+      </c>
+      <c r="H35" s="20" t="n">
+        <v>127.9943914724202</v>
+      </c>
+      <c r="I35" s="20" t="n">
+        <v>92.12685245600574</v>
+      </c>
+      <c r="J35" s="21" t="n">
+        <v>0.9896395277597415</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2024-08-31</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="n">
+        <v>1169785</v>
+      </c>
+      <c r="C36" s="18" t="n">
+        <v>78803000</v>
+      </c>
+      <c r="D36" s="18" t="n">
+        <v>79972785</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="19" t="n">
+        <v>-0.05165383522819074</v>
+      </c>
+      <c r="G36" s="19" t="n">
+        <v>-0.03721446516187343</v>
+      </c>
+      <c r="H36" s="20" t="n">
+        <v>121.3829902651713</v>
+      </c>
+      <c r="I36" s="20" t="n">
+        <v>88.69840091480866</v>
+      </c>
+      <c r="J36" s="21" t="n">
+        <v>0.9853727114792864</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="B37" s="18" t="n">
+        <v>1169785</v>
+      </c>
+      <c r="C37" s="18" t="n">
+        <v>81306000</v>
+      </c>
+      <c r="D37" s="18" t="n">
+        <v>82475785</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="19" t="n">
+        <v>0.03129814723846368</v>
+      </c>
+      <c r="G37" s="19" t="n">
+        <v>-0.03030315755724822</v>
+      </c>
+      <c r="H37" s="20" t="n">
+        <v>125.1820529667356</v>
+      </c>
+      <c r="I37" s="20" t="n">
+        <v>86.01055929681125</v>
+      </c>
+      <c r="J37" s="21" t="n">
+        <v>0.9858166248432798</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2024-10-31</t>
+        </is>
+      </c>
+      <c r="B38" s="18" t="n">
+        <v>28260879</v>
+      </c>
+      <c r="C38" s="18" t="n">
+        <v>54002000</v>
+      </c>
+      <c r="D38" s="18" t="n">
+        <v>82262879</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="19" t="n">
+        <v>-0.00258143647859793</v>
+      </c>
+      <c r="G38" s="19" t="n">
+        <v>-0.01963155079337908</v>
+      </c>
+      <c r="H38" s="20" t="n">
+        <v>124.8589034487415</v>
+      </c>
+      <c r="I38" s="20" t="n">
+        <v>84.32203863320896</v>
+      </c>
+      <c r="J38" s="21" t="n">
+        <v>0.6564564802065826</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2024-11-30</t>
+        </is>
+      </c>
+      <c r="B39" s="18" t="n">
+        <v>40410525</v>
+      </c>
+      <c r="C39" s="18" t="n">
+        <v>54680000</v>
+      </c>
+      <c r="D39" s="18" t="n">
+        <v>95090525</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="19" t="n">
+        <v>0.1559348050534434</v>
+      </c>
+      <c r="G39" s="19" t="n">
+        <v>-0.0340039143393287</v>
+      </c>
+      <c r="H39" s="20" t="n">
+        <v>144.3287522172077</v>
+      </c>
+      <c r="I39" s="20" t="n">
+        <v>81.45475925460775</v>
+      </c>
+      <c r="J39" s="21" t="n">
+        <v>0.5750310033518061</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
+      </c>
+      <c r="B40" s="18" t="n">
+        <v>51289275</v>
+      </c>
+      <c r="C40" s="18" t="n">
+        <v>50030000</v>
+      </c>
+      <c r="D40" s="18" t="n">
+        <v>101319275</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="19" t="n">
+        <v>0.06550337165558819</v>
+      </c>
+      <c r="G40" s="19" t="n">
+        <v>-0.02297312356483838</v>
+      </c>
+      <c r="H40" s="20" t="n">
+        <v>153.7827721142787</v>
+      </c>
+      <c r="I40" s="20" t="n">
+        <v>79.58348900530748</v>
+      </c>
+      <c r="J40" s="21" t="n">
+        <v>0.493785609895057</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-01-31</t>
+        </is>
+      </c>
+      <c r="B41" s="18" t="n">
+        <v>17052502</v>
+      </c>
+      <c r="C41" s="18" t="n">
+        <v>83500000</v>
+      </c>
+      <c r="D41" s="18" t="n">
+        <v>100552502</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="19" t="n">
+        <v>-0.007567888735879723</v>
+      </c>
+      <c r="G41" s="19" t="n">
+        <v>0.04912715928504907</v>
+      </c>
+      <c r="H41" s="20" t="n">
+        <v>152.6189612054227</v>
+      </c>
+      <c r="I41" s="20" t="n">
+        <v>83.49319974613117</v>
+      </c>
+      <c r="J41" s="21" t="n">
+        <v>0.8304119573275263</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="n">
+        <v>17052502</v>
+      </c>
+      <c r="C42" s="18" t="n">
+        <v>84100000</v>
+      </c>
+      <c r="D42" s="18" t="n">
+        <v>101152502</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="19" t="n">
+        <v>0.005967032028700788</v>
+      </c>
+      <c r="G42" s="19" t="n">
+        <v>0.006121432841425634</v>
+      </c>
+      <c r="H42" s="20" t="n">
+        <v>153.5296434351225</v>
+      </c>
+      <c r="I42" s="20" t="n">
+        <v>84.00429776109284</v>
+      </c>
+      <c r="J42" s="21" t="n">
+        <v>0.8314178921644469</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="n">
+        <v>17052502</v>
+      </c>
+      <c r="C43" s="18" t="n">
+        <v>87900000</v>
+      </c>
+      <c r="D43" s="18" t="n">
+        <v>104952502</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="19" t="n">
+        <v>0.0375670391227693</v>
+      </c>
+      <c r="G43" s="19" t="n">
+        <v>-0.004497088806370564</v>
+      </c>
+      <c r="H43" s="20" t="n">
+        <v>159.2972975565546</v>
+      </c>
+      <c r="I43" s="20" t="n">
+        <v>83.62652297394442</v>
+      </c>
+      <c r="J43" s="21" t="n">
+        <v>0.8375217200634245</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-04-30</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="n">
+        <v>17428114</v>
+      </c>
+      <c r="C44" s="18" t="n">
+        <v>95700000</v>
+      </c>
+      <c r="D44" s="18" t="n">
+        <v>113128114</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="19" t="n">
+        <v>0.07789820961104862</v>
+      </c>
+      <c r="G44" s="19" t="n">
+        <v>0.01396857144046737</v>
+      </c>
+      <c r="H44" s="20" t="n">
+        <v>171.7062718320887</v>
+      </c>
+      <c r="I44" s="20" t="n">
+        <v>84.79466603442386</v>
+      </c>
+      <c r="J44" s="21" t="n">
+        <v>0.8459435644794715</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-05-31</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="n">
+        <v>2736904</v>
+      </c>
+      <c r="C45" s="18" t="n">
+        <v>96750000</v>
+      </c>
+      <c r="D45" s="18" t="n">
+        <v>99486904</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>-15000000</v>
+      </c>
+      <c r="F45" s="19" t="n">
+        <v>0.01254776502373523</v>
+      </c>
+      <c r="G45" s="19" t="n">
+        <v>0.05517455088033429</v>
+      </c>
+      <c r="H45" s="20" t="n">
+        <v>173.8608017841393</v>
+      </c>
+      <c r="I45" s="20" t="n">
+        <v>89.47317364992112</v>
+      </c>
+      <c r="J45" s="21" t="n">
+        <v>0.9724898062965152</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="B46" s="18" t="n">
+        <v>2736904</v>
+      </c>
+      <c r="C46" s="18" t="n">
+        <v>102250000</v>
+      </c>
+      <c r="D46" s="18" t="n">
+        <v>104986904</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="19" t="n">
+        <v>0.05528365823907838</v>
+      </c>
+      <c r="G46" s="19" t="n">
+        <v>0.1453031659990138</v>
+      </c>
+      <c r="H46" s="20" t="n">
+        <v>183.4724629311458</v>
+      </c>
+      <c r="I46" s="20" t="n">
+        <v>102.4739090532342</v>
+      </c>
+      <c r="J46" s="21" t="n">
+        <v>0.9739309961935824</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="n">
+        <v>2746705</v>
+      </c>
+      <c r="C47" s="18" t="n">
+        <v>116550000</v>
+      </c>
+      <c r="D47" s="18" t="n">
+        <v>119296705</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="19" t="n">
+        <v>0.1363008190050066</v>
+      </c>
+      <c r="G47" s="19" t="n">
+        <v>0.009632162447612558</v>
+      </c>
+      <c r="H47" s="20" t="n">
+        <v>208.4799098935267</v>
+      </c>
+      <c r="I47" s="20" t="n">
+        <v>103.4609543918768</v>
+      </c>
+      <c r="J47" s="21" t="n">
+        <v>0.9769758519315349</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-08-31</t>
+        </is>
+      </c>
+      <c r="B48" s="18" t="n">
+        <v>11521868</v>
+      </c>
+      <c r="C48" s="18" t="n">
+        <v>91434000</v>
+      </c>
+      <c r="D48" s="18" t="n">
+        <v>102955868</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>-20000000</v>
+      </c>
+      <c r="F48" s="19" t="n">
+        <v>0.03117863775443296</v>
+      </c>
+      <c r="G48" s="19" t="n">
+        <v>0.007539893824132227</v>
+      </c>
+      <c r="H48" s="20" t="n">
+        <v>214.9800294831738</v>
+      </c>
+      <c r="I48" s="20" t="n">
+        <v>104.241039002935</v>
+      </c>
+      <c r="J48" s="21" t="n">
+        <v>0.8880892539315972</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="n">
+        <v>14007763</v>
+      </c>
+      <c r="C49" s="18" t="n">
+        <v>101760000</v>
+      </c>
+      <c r="D49" s="18" t="n">
+        <v>115767763</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="19" t="n">
+        <v>0.1244406486864838</v>
+      </c>
+      <c r="G49" s="19" t="n">
+        <v>0.09955683177481456</v>
+      </c>
+      <c r="H49" s="20" t="n">
+        <v>241.7322838066993</v>
+      </c>
+      <c r="I49" s="20" t="n">
+        <v>114.618946586982</v>
+      </c>
+      <c r="J49" s="21" t="n">
+        <v>0.8790011775557933</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2025-10-31</t>
+        </is>
+      </c>
+      <c r="B50" s="18" t="n">
+        <v>14020365</v>
+      </c>
+      <c r="C50" s="18" t="n">
+        <v>121500000</v>
+      </c>
+      <c r="D50" s="18" t="n">
+        <v>135520365</v>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="19" t="n">
+        <v>0.1706226456150837</v>
+      </c>
+      <c r="G50" s="19" t="n">
+        <v>0.1885711702088579</v>
+      </c>
+      <c r="H50" s="20" t="n">
+        <v>282.9772856003746</v>
+      </c>
+      <c r="I50" s="20" t="n">
+        <v>136.2327754729958</v>
+      </c>
+      <c r="J50" s="21" t="n">
+        <v>0.8965442204940932</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="n">
+        <v>14289845</v>
+      </c>
+      <c r="C51" s="18" t="n">
+        <v>109405000</v>
+      </c>
+      <c r="D51" s="18" t="n">
+        <v>123694845</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="19" t="n">
+        <v>-0.08726009555833177</v>
+      </c>
+      <c r="G51" s="19" t="n">
+        <v>-0.0455580968502739</v>
+      </c>
+      <c r="H51" s="20" t="n">
+        <v>258.2846606180486</v>
+      </c>
+      <c r="I51" s="20" t="n">
+        <v>130.0262694938155</v>
+      </c>
+      <c r="J51" s="21" t="n">
+        <v>0.8844750159151742</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="n">
+        <v>14289845</v>
+      </c>
+      <c r="C52" s="18" t="n">
+        <v>120295000</v>
+      </c>
+      <c r="D52" s="18" t="n">
+        <v>134584845</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="19" t="n">
+        <v>0.08803923882195737</v>
+      </c>
+      <c r="G52" s="19" t="n">
+        <v>0.07494185393349384</v>
+      </c>
+      <c r="H52" s="20" t="n">
+        <v>281.0238455382491</v>
+      </c>
+      <c r="I52" s="20" t="n">
+        <v>139.7706791897381</v>
+      </c>
+      <c r="J52" s="21" t="n">
+        <v>0.8938227777429175</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B53" s="18" t="n">
+        <v>1459510</v>
+      </c>
+      <c r="C53" s="18" t="n">
+        <v>166095000</v>
+      </c>
+      <c r="D53" s="18" t="n">
+        <v>167554510</v>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="19" t="n">
+        <v>0.2449730874230304</v>
+      </c>
+      <c r="G53" s="19" t="n">
+        <v>0.2397126741763627</v>
+      </c>
+      <c r="H53" s="20" t="n">
+        <v>349.8671246192469</v>
+      </c>
+      <c r="I53" s="20" t="n">
+        <v>173.2754824697567</v>
+      </c>
+      <c r="J53" s="21" t="n">
+        <v>0.9912893421967574</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B54" s="18" t="n">
+        <v>1459510</v>
+      </c>
+      <c r="C54" s="18" t="n">
+        <v>221895000</v>
+      </c>
+      <c r="D54" s="18" t="n">
+        <v>223354510</v>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="19" t="n">
+        <v>0.3330259507786451</v>
+      </c>
+      <c r="G54" s="19" t="n">
+        <v>0.1951952097899254</v>
+      </c>
+      <c r="H54" s="20" t="n">
+        <v>466.3819564417622</v>
+      </c>
+      <c r="I54" s="20" t="n">
+        <v>207.0980266218914</v>
+      </c>
+      <c r="J54" s="21" t="n">
+        <v>0.9934655002041374</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B55" s="18" t="n">
+        <v>25341</v>
+      </c>
+      <c r="C55" s="18" t="n">
+        <v>150225600</v>
+      </c>
+      <c r="D55" s="18" t="n">
+        <v>150250941</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>-49999999</v>
+      </c>
+      <c r="F55" s="19" t="n">
+        <v>-0.1041914069837425</v>
+      </c>
+      <c r="G55" s="19" t="n">
+        <v>-0.1225838830814379</v>
+      </c>
+      <c r="H55" s="20" t="n">
+        <v>417.7889642082645</v>
+      </c>
+      <c r="I55" s="20" t="n">
+        <v>181.711146340077</v>
+      </c>
+      <c r="J55" s="21" t="n">
+        <v>0.9998313421544561</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B56" s="18" t="n">
+        <v>901285</v>
+      </c>
+      <c r="C56" s="18" t="n">
+        <v>162085000</v>
+      </c>
+      <c r="D56" s="18" t="n">
+        <v>162986285</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="19" t="n">
+        <v>0.08476049411231308</v>
+      </c>
+      <c r="G56" s="19" t="n">
+        <v>0.2044590654610745</v>
+      </c>
+      <c r="H56" s="20" t="n">
+        <v>453.2009632492285</v>
+      </c>
+      <c r="I56" s="20" t="n">
+        <v>218.8636375046297</v>
+      </c>
+      <c r="J56" s="21" t="n">
+        <v>0.9944701788865241</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B57" s="18" t="n">
+        <v>1153815</v>
+      </c>
+      <c r="C57" s="18" t="n">
+        <v>204330000</v>
+      </c>
+      <c r="D57" s="18" t="n">
+        <v>205483815</v>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="19" t="n">
+        <v>0.2607429821472402</v>
+      </c>
+      <c r="G57" s="19" t="n">
+        <v>0.3318007062939723</v>
+      </c>
+      <c r="H57" s="20" t="n">
+        <v>571.3699339188341</v>
+      </c>
+      <c r="I57" s="20" t="n">
+        <v>291.4827470107338</v>
+      </c>
+      <c r="J57" s="21" t="n">
+        <v>0.9943848862257108</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B58" s="18" t="n">
+        <v>61652155</v>
+      </c>
+      <c r="C58" s="18" t="n">
+        <v>125800000</v>
+      </c>
+      <c r="D58" s="18" t="n">
+        <v>187452155</v>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="19" t="n">
+        <v>-0.08775221542387657</v>
+      </c>
+      <c r="G58" s="19" t="n">
+        <v>-0.0551830636623889</v>
+      </c>
+      <c r="H58" s="20" t="n">
+        <v>521.2309563908625</v>
+      </c>
+      <c r="I58" s="20" t="n">
+        <v>275.3978360259524</v>
+      </c>
+      <c r="J58" s="21" t="n">
+        <v>0.6711045813263656</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B59" s="18" t="n">
+        <v>61675133</v>
+      </c>
+      <c r="C59" s="18" t="n">
+        <v>105000000</v>
+      </c>
+      <c r="D59" s="18" t="n">
+        <v>166675133</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="19" t="n">
+        <v>-0.1108390671742344</v>
+      </c>
+      <c r="G59" s="19" t="n">
+        <v>-0.2056937967410791</v>
+      </c>
+      <c r="H59" s="20" t="n">
+        <v>463.4582034021652</v>
+      </c>
+      <c r="I59" s="20" t="n">
+        <v>218.7502095194971</v>
+      </c>
+      <c r="J59" s="21" t="n">
+        <v>0.6299679988855926</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B60" s="18" t="n">
+        <v>61801703</v>
+      </c>
+      <c r="C60" s="18" t="n">
+        <v>104400000</v>
+      </c>
+      <c r="D60" s="18" t="n">
+        <v>166201703</v>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="19" t="n">
+        <v>-0.002840435711546725</v>
+      </c>
+      <c r="G60" s="19" t="n">
+        <v>0.03644172910983712</v>
+      </c>
+      <c r="H60" s="20" t="n">
+        <v>462.1417801704125</v>
+      </c>
+      <c r="I60" s="20" t="n">
+        <v>226.7218453975268</v>
+      </c>
+      <c r="J60" s="21" t="n">
+        <v>0.6281524082818815</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="n">
+        <v>61801703</v>
+      </c>
+      <c r="C61" s="18" t="n">
+        <v>110400000</v>
+      </c>
+      <c r="D61" s="18" t="n">
+        <v>172201703</v>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="19" t="n">
+        <v>0.03610071311964836</v>
+      </c>
+      <c r="G61" s="19" t="n">
+        <v>0.01982947085077003</v>
+      </c>
+      <c r="H61" s="20" t="n">
+        <v>478.8254279969482</v>
+      </c>
+      <c r="I61" s="20" t="n">
+        <v>231.2176196220698</v>
+      </c>
+      <c r="J61" s="21" t="n">
+        <v>0.6411086422298623</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B62" s="18" t="n">
+        <v>61879843</v>
+      </c>
+      <c r="C62" s="18" t="n">
+        <v>95000000</v>
+      </c>
+      <c r="D62" s="18" t="n">
+        <v>156879843</v>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="19" t="n">
+        <v>-0.08897623968329745</v>
+      </c>
+      <c r="G62" s="19" t="n">
+        <v>-0.1260444796206572</v>
+      </c>
+      <c r="H62" s="20" t="n">
+        <v>436.2213419490342</v>
+      </c>
+      <c r="I62" s="20" t="n">
+        <v>202.073915077679</v>
+      </c>
+      <c r="J62" s="21" t="n">
+        <v>0.6055589945994527</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1152,10 +3386,10 @@
         <v>1450840</v>
       </c>
       <c r="J2" s="10" t="n">
-        <v>22601414.76425532</v>
+        <v>22001414.76425532</v>
       </c>
       <c r="K2" s="10" t="n">
-        <v>106121184</v>
+        <v>105521184</v>
       </c>
     </row>
     <row r="3">
@@ -1319,7 +3553,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3549,7 +5783,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3637,16 +5871,16 @@
         <v>72998585.23574468</v>
       </c>
       <c r="F2" s="10" t="n">
-        <v>239000</v>
+        <v>237500</v>
       </c>
       <c r="G2" s="10" t="n">
-        <v>95600000</v>
+        <v>95000000</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>22601414.76425532</v>
+        <v>22001414.76425532</v>
       </c>
       <c r="I2" s="14" t="n">
-        <v>0.3096144218585245</v>
+        <v>0.3013950844828434</v>
       </c>
     </row>
   </sheetData>
@@ -3654,7 +5888,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4799,7 +7033,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>